<commit_message>
feat(batch): refine Paper 384 exclusion to Code 6 Duplicate and populate verbatim evidence for batch 383-389
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/383_384_385_387_389.xlsx
+++ b/03_Coding_Sheets/383_384_385_387_389.xlsx
@@ -6309,7 +6309,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>1 = No effect size of interest</t>
+          <t>6 = Duplicate / retracted</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>The study uses an identical sample (N=170 product managers from Fortune 500 consumer packaged goods industries) and reports the exact same correlation values as Paper [383] (Lysonski, 1985 in Journal of Marketing). Sliced duplicate publication cited directly in Endnote 6 (p. 26). Excluded under Code 6 (Duplicate) to prevent double counting in meta-analysis. Verbatim Evidence: [p. 18] "Questionnaires were mailed to 449 product managers in consumer packaged goods industries, drawn from the Fortune 500.6 The sampled industries included food, proprietary drugs and cosmetics, soaps, cleansers and allied products, soft drinks, tobacco, paper, and liquor. All of these industries have been using product managers for many years. The final usable sample was 170 completed questionnaires." [p. 26] "6. Lysonski, S., 'A Boundary Theory Investigation of the Product Manager's Role,' Journal of Marketing, 49, (1985), 26-40."</t>
         </is>
       </c>
     </row>
@@ -6332,6 +6337,11 @@
           <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Data collected from individual respondents were aggregated to the team level of analysis (N = 23 teams) to examine hypotheses regarding team-level outcomes; no individual-level correlation matrix is reported. Verbatim Evidence: [p. 4] "The final sample consisted of 83 team members and team managers from 23 teams located in the United States and India." [p. 48] "Data collected from individual respondents were aggregated to the team level of analysis (N = 23 teams) to examine the hypotheses regarding team-level outcomes."</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6352,6 +6362,11 @@
           <t>1 = No effect size of interest</t>
         </is>
       </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Boundary spanning was operationalized solely as generative AI tool usage (querying ChatGPT and AI tools for external information acquisition) rather than interpersonal or cross-unit boundary spanning. Table 4 reports PLS-SEM latent correlations but lacks zero-order Pearson correlations and descriptive statistics (Mean/SD). Excluded under Code 1 per AI Tool Interaction trap. Verbatim Evidence: [Table 2, p. 7] "I use AI tools to solicit information and resources from external channels." "I make use of external resources through AI tools to support my work." "I actively use AI tools to solicit external work resources." "My work depends upon information and resources actively solicited through AI tools, that is, information and resources beyond those coming through official channels."</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6370,6 +6385,11 @@
       <c r="F47" t="inlineStr">
         <is>
           <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>The focal unit of statistical analysis is collaborative project teams (N = 452). Survey items use the team as the grammatical referent, violating the individual worker analysis requirement. Verbatim Evidence: [p. 62] "The unit of analysis for this study is the collaborative project team (N = 452 project teams across engineering and construction sectors)." [p. 67] "All survey items were worded with the team as the referent, for example, 'The team actively reaches out to external stakeholders to coordinate project delivery.'"</t>
         </is>
       </c>
     </row>

</xml_diff>